<commit_message>
Update GPU configuration and benchmark results
</commit_message>
<xml_diff>
--- a/results_final/benchmark_summary.xlsx
+++ b/results_final/benchmark_summary.xlsx
@@ -549,16 +549,16 @@
         <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>15.0483</v>
+        <v>13.835</v>
       </c>
       <c r="H2" t="n">
         <v>107195</v>
       </c>
       <c r="I2" t="n">
-        <v>0.033064</v>
+        <v>0.0276</v>
       </c>
       <c r="J2" t="n">
-        <v>239.2</v>
+        <v>260.2</v>
       </c>
       <c r="K2" t="n">
         <v>43.4</v>
@@ -573,10 +573,10 @@
         <v>35.4</v>
       </c>
       <c r="O2" t="n">
-        <v>28.6858</v>
+        <v>30.8133</v>
       </c>
       <c r="P2" t="n">
-        <v>2.7553</v>
+        <v>2.3</v>
       </c>
       <c r="Q2" t="n">
         <v>66.7</v>
@@ -598,54 +598,54 @@
         <v>12</v>
       </c>
       <c r="C3" t="n">
-        <v>50.1</v>
+        <v>50.2</v>
       </c>
       <c r="D3" t="n">
         <v>24.5</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>86.1% pool recall</t>
+          <t>88.9% pool recall</t>
         </is>
       </c>
       <c r="F3" t="n">
         <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>4.8435</v>
+        <v>4.7307</v>
       </c>
       <c r="H3" t="n">
-        <v>287585</v>
+        <v>287625</v>
       </c>
       <c r="I3" t="n">
-        <v>0.018997</v>
+        <v>0.018847</v>
       </c>
       <c r="J3" t="n">
-        <v>743.3</v>
+        <v>761</v>
       </c>
       <c r="K3" t="n">
-        <v>53.2</v>
+        <v>55.1</v>
       </c>
       <c r="L3" t="n">
-        <v>29</v>
+        <v>28.6</v>
       </c>
       <c r="M3" t="n">
-        <v>24.4</v>
+        <v>25.3</v>
       </c>
       <c r="N3" t="n">
         <v>33.3</v>
       </c>
       <c r="O3" t="n">
-        <v>85.3167</v>
+        <v>90.4967</v>
       </c>
       <c r="P3" t="n">
-        <v>1.5831</v>
+        <v>1.5706</v>
       </c>
       <c r="Q3" t="n">
         <v>83.3</v>
       </c>
       <c r="R3" t="n">
-        <v>16.9</v>
+        <v>17.1</v>
       </c>
       <c r="S3" t="n">
         <v>44.4</v>

</xml_diff>

<commit_message>
Add Docker setup and update dependencies
</commit_message>
<xml_diff>
--- a/results_final/benchmark_summary.xlsx
+++ b/results_final/benchmark_summary.xlsx
@@ -549,16 +549,16 @@
         <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>13.835</v>
+        <v>13.6569</v>
       </c>
       <c r="H2" t="n">
         <v>107195</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0276</v>
+        <v>0.027856</v>
       </c>
       <c r="J2" t="n">
-        <v>260.2</v>
+        <v>263.6</v>
       </c>
       <c r="K2" t="n">
         <v>43.4</v>
@@ -573,10 +573,10 @@
         <v>35.4</v>
       </c>
       <c r="O2" t="n">
-        <v>30.8133</v>
+        <v>31.1258</v>
       </c>
       <c r="P2" t="n">
-        <v>2.3</v>
+        <v>2.3213</v>
       </c>
       <c r="Q2" t="n">
         <v>66.7</v>
@@ -598,57 +598,57 @@
         <v>12</v>
       </c>
       <c r="C3" t="n">
-        <v>50.2</v>
+        <v>49.1</v>
       </c>
       <c r="D3" t="n">
-        <v>24.5</v>
+        <v>26.4</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>88.9% pool recall</t>
+          <t>86.1% pool recall</t>
         </is>
       </c>
       <c r="F3" t="n">
         <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>4.7307</v>
+        <v>4.6067</v>
       </c>
       <c r="H3" t="n">
-        <v>287625</v>
+        <v>287581</v>
       </c>
       <c r="I3" t="n">
-        <v>0.018847</v>
+        <v>0.016684</v>
       </c>
       <c r="J3" t="n">
-        <v>761</v>
+        <v>781.5</v>
       </c>
       <c r="K3" t="n">
-        <v>55.1</v>
+        <v>50.4</v>
       </c>
       <c r="L3" t="n">
-        <v>28.6</v>
+        <v>25.9</v>
       </c>
       <c r="M3" t="n">
-        <v>25.3</v>
+        <v>21.9</v>
       </c>
       <c r="N3" t="n">
-        <v>33.3</v>
+        <v>35.4</v>
       </c>
       <c r="O3" t="n">
-        <v>90.4967</v>
+        <v>95.3967</v>
       </c>
       <c r="P3" t="n">
-        <v>1.5706</v>
+        <v>1.3903</v>
       </c>
       <c r="Q3" t="n">
         <v>83.3</v>
       </c>
       <c r="R3" t="n">
-        <v>17.1</v>
+        <v>14.9</v>
       </c>
       <c r="S3" t="n">
-        <v>44.4</v>
+        <v>47.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AsyncLLMEngine + Docker benchmark — all metrics passing
</commit_message>
<xml_diff>
--- a/results_final/benchmark_summary.xlsx
+++ b/results_final/benchmark_summary.xlsx
@@ -549,16 +549,16 @@
         <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>13.6569</v>
+        <v>13.1073</v>
       </c>
       <c r="H2" t="n">
         <v>107195</v>
       </c>
       <c r="I2" t="n">
-        <v>0.027856</v>
+        <v>0.024829</v>
       </c>
       <c r="J2" t="n">
-        <v>263.6</v>
+        <v>274.7</v>
       </c>
       <c r="K2" t="n">
         <v>43.4</v>
@@ -573,10 +573,10 @@
         <v>35.4</v>
       </c>
       <c r="O2" t="n">
-        <v>31.1258</v>
+        <v>32.2317</v>
       </c>
       <c r="P2" t="n">
-        <v>2.3213</v>
+        <v>2.0691</v>
       </c>
       <c r="Q2" t="n">
         <v>66.7</v>
@@ -598,10 +598,10 @@
         <v>12</v>
       </c>
       <c r="C3" t="n">
-        <v>49.1</v>
+        <v>50</v>
       </c>
       <c r="D3" t="n">
-        <v>26.4</v>
+        <v>31.3</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -612,43 +612,43 @@
         <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>4.6067</v>
+        <v>4.618</v>
       </c>
       <c r="H3" t="n">
-        <v>287581</v>
+        <v>287633</v>
       </c>
       <c r="I3" t="n">
-        <v>0.016684</v>
+        <v>0.018379</v>
       </c>
       <c r="J3" t="n">
-        <v>781.5</v>
+        <v>779.6</v>
       </c>
       <c r="K3" t="n">
-        <v>50.4</v>
+        <v>54.3</v>
       </c>
       <c r="L3" t="n">
-        <v>25.9</v>
+        <v>29.1</v>
       </c>
       <c r="M3" t="n">
-        <v>21.9</v>
+        <v>24.4</v>
       </c>
       <c r="N3" t="n">
-        <v>35.4</v>
+        <v>39.6</v>
       </c>
       <c r="O3" t="n">
-        <v>95.3967</v>
+        <v>90.4842</v>
       </c>
       <c r="P3" t="n">
-        <v>1.3903</v>
+        <v>1.5316</v>
       </c>
       <c r="Q3" t="n">
         <v>83.3</v>
       </c>
       <c r="R3" t="n">
-        <v>14.9</v>
+        <v>16.8</v>
       </c>
       <c r="S3" t="n">
-        <v>47.2</v>
+        <v>52.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
native+docker+k8s benchmarks, AsyncLLMEngine, Prometheus+Grafana initial
</commit_message>
<xml_diff>
--- a/results_final/benchmark_summary.xlsx
+++ b/results_final/benchmark_summary.xlsx
@@ -549,16 +549,16 @@
         <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>13.1073</v>
+        <v>13.1277</v>
       </c>
       <c r="H2" t="n">
         <v>107195</v>
       </c>
       <c r="I2" t="n">
-        <v>0.024829</v>
+        <v>0.056131</v>
       </c>
       <c r="J2" t="n">
-        <v>274.7</v>
+        <v>274.2</v>
       </c>
       <c r="K2" t="n">
         <v>43.4</v>
@@ -573,10 +573,10 @@
         <v>35.4</v>
       </c>
       <c r="O2" t="n">
-        <v>32.2317</v>
+        <v>32.1225</v>
       </c>
       <c r="P2" t="n">
-        <v>2.0691</v>
+        <v>4.6776</v>
       </c>
       <c r="Q2" t="n">
         <v>66.7</v>
@@ -598,57 +598,57 @@
         <v>12</v>
       </c>
       <c r="C3" t="n">
-        <v>50</v>
+        <v>53.6</v>
       </c>
       <c r="D3" t="n">
-        <v>31.3</v>
+        <v>26.4</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>86.1% pool recall</t>
+          <t>88.9% pool recall</t>
         </is>
       </c>
       <c r="F3" t="n">
         <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>4.618</v>
+        <v>4.3042</v>
       </c>
       <c r="H3" t="n">
-        <v>287633</v>
+        <v>287482</v>
       </c>
       <c r="I3" t="n">
-        <v>0.018379</v>
+        <v>0.072424</v>
       </c>
       <c r="J3" t="n">
-        <v>779.6</v>
+        <v>836.4</v>
       </c>
       <c r="K3" t="n">
-        <v>54.3</v>
+        <v>51.5</v>
       </c>
       <c r="L3" t="n">
-        <v>29.1</v>
+        <v>27</v>
       </c>
       <c r="M3" t="n">
-        <v>24.4</v>
+        <v>22.8</v>
       </c>
       <c r="N3" t="n">
-        <v>39.6</v>
+        <v>35.4</v>
       </c>
       <c r="O3" t="n">
-        <v>90.4842</v>
+        <v>96.46080000000001</v>
       </c>
       <c r="P3" t="n">
-        <v>1.5316</v>
+        <v>6.0353</v>
       </c>
       <c r="Q3" t="n">
-        <v>83.3</v>
+        <v>91.7</v>
       </c>
       <c r="R3" t="n">
-        <v>16.8</v>
+        <v>15.6</v>
       </c>
       <c r="S3" t="n">
-        <v>52.8</v>
+        <v>47.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finalize benchmark metrics and deployment
</commit_message>
<xml_diff>
--- a/results_final/benchmark_summary.xlsx
+++ b/results_final/benchmark_summary.xlsx
@@ -549,16 +549,16 @@
         <v>100</v>
       </c>
       <c r="G2" t="n">
-        <v>13.1277</v>
+        <v>56.3916</v>
       </c>
       <c r="H2" t="n">
         <v>107195</v>
       </c>
       <c r="I2" t="n">
-        <v>0.056131</v>
+        <v>0.057493</v>
       </c>
       <c r="J2" t="n">
-        <v>274.2</v>
+        <v>63.8</v>
       </c>
       <c r="K2" t="n">
         <v>43.4</v>
@@ -573,10 +573,10 @@
         <v>35.4</v>
       </c>
       <c r="O2" t="n">
-        <v>32.1225</v>
+        <v>29.1592</v>
       </c>
       <c r="P2" t="n">
-        <v>4.6776</v>
+        <v>4.7911</v>
       </c>
       <c r="Q2" t="n">
         <v>66.7</v>
@@ -598,57 +598,57 @@
         <v>12</v>
       </c>
       <c r="C3" t="n">
-        <v>53.6</v>
+        <v>50.1</v>
       </c>
       <c r="D3" t="n">
-        <v>26.4</v>
+        <v>24.5</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>88.9% pool recall</t>
+          <t>86.1% pool recall</t>
         </is>
       </c>
       <c r="F3" t="n">
         <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>4.3042</v>
+        <v>71.9817</v>
       </c>
       <c r="H3" t="n">
-        <v>287482</v>
+        <v>287621</v>
       </c>
       <c r="I3" t="n">
-        <v>0.072424</v>
+        <v>0.07462100000000001</v>
       </c>
       <c r="J3" t="n">
-        <v>836.4</v>
+        <v>50</v>
       </c>
       <c r="K3" t="n">
-        <v>51.5</v>
+        <v>53.4</v>
       </c>
       <c r="L3" t="n">
-        <v>27</v>
+        <v>29.1</v>
       </c>
       <c r="M3" t="n">
-        <v>22.8</v>
+        <v>24.4</v>
       </c>
       <c r="N3" t="n">
-        <v>35.4</v>
+        <v>33.3</v>
       </c>
       <c r="O3" t="n">
-        <v>96.46080000000001</v>
+        <v>105.6742</v>
       </c>
       <c r="P3" t="n">
-        <v>6.0353</v>
+        <v>6.2184</v>
       </c>
       <c r="Q3" t="n">
-        <v>91.7</v>
+        <v>83.3</v>
       </c>
       <c r="R3" t="n">
-        <v>15.6</v>
+        <v>16.9</v>
       </c>
       <c r="S3" t="n">
-        <v>47.2</v>
+        <v>44.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>